<commit_message>
feat: complete bulk import with built-in CSV/XLSX templates for student, teacher, and admin on corresponding pages
</commit_message>
<xml_diff>
--- a/public/templates/student_upload_template.xlsx
+++ b/public/templates/student_upload_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Students" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -442,43 +442,43 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Jimmy</v>
+        <v>Arun</v>
       </c>
       <c r="B2" t="str">
-        <v>Doe</v>
+        <v>Kumar</v>
       </c>
       <c r="C2" t="str">
-        <v>101</v>
+        <v>2025CS101</v>
       </c>
       <c r="D2" t="str">
-        <v>ADM101</v>
+        <v>ADM-2025-001</v>
       </c>
       <c r="E2" t="str">
         <v>2010-05-15</v>
       </c>
       <c r="F2" t="str">
-        <v>Class 1 - A</v>
+        <v>Class 10 - A</v>
       </c>
       <c r="G2" t="str">
-        <v>Dayscholar (or Hostel)</v>
+        <v>DAYSCHOLAR</v>
       </c>
       <c r="H2" t="str">
-        <v>Jane</v>
+        <v>Ramesh</v>
       </c>
       <c r="I2" t="str">
-        <v>Doe</v>
+        <v>Kumar</v>
       </c>
       <c r="J2" t="str">
-        <v>jane.parent@example.com</v>
+        <v>ramesh.parent@example.com</v>
       </c>
       <c r="K2" t="str">
-        <v>password123</v>
+        <v>Parent@123</v>
       </c>
       <c r="L2" t="str">
         <v>9876543210</v>
       </c>
       <c r="M2" t="str">
-        <v>123 Main Street</v>
+        <v>123 Park Street, City</v>
       </c>
     </row>
   </sheetData>

</xml_diff>